<commit_message>
Reinstall venv and refactor mechanism python
</commit_message>
<xml_diff>
--- a/Backend/dataset/KandunganGiziProduct.xlsx
+++ b/Backend/dataset/KandunganGiziProduct.xlsx
@@ -37,22 +37,22 @@
     <t>Ukuran (ml)</t>
   </si>
   <si>
-    <t>Energi (kcal/100g)</t>
-  </si>
-  <si>
-    <t>Gula (g/100g)</t>
-  </si>
-  <si>
-    <t>Garam/Natrium (g/100g)</t>
-  </si>
-  <si>
-    <t>Lemak (g/100g)</t>
-  </si>
-  <si>
-    <t>Protein (g/100g)</t>
-  </si>
-  <si>
-    <t>Karbohidrat (g/100g)</t>
+    <t>Energi (g)</t>
+  </si>
+  <si>
+    <t>Gula (g)</t>
+  </si>
+  <si>
+    <t>Garam/Natrium (g)</t>
+  </si>
+  <si>
+    <t>Lemak (g)</t>
+  </si>
+  <si>
+    <t>Protein (g)</t>
+  </si>
+  <si>
+    <t>Karbohidrat (g)</t>
   </si>
   <si>
     <t>Grade</t>
@@ -601,7 +601,7 @@
     <col customWidth="1" min="2" max="2" width="27.75"/>
     <col customWidth="1" min="3" max="4" width="30.88"/>
     <col customWidth="1" min="6" max="6" width="23.38"/>
-    <col customWidth="1" min="7" max="7" width="135.25"/>
+    <col customWidth="1" min="7" max="7" width="229.38"/>
     <col customWidth="1" min="9" max="9" width="20.13"/>
     <col customWidth="1" min="10" max="10" width="21.0"/>
     <col customWidth="1" min="11" max="11" width="21.75"/>

</xml_diff>